<commit_message>
remove global GHG market
</commit_message>
<xml_diff>
--- a/tasks.xlsx
+++ b/tasks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\GCAM-CDR-policy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CC473DC-8547-46B8-8CA5-CDF98634A556}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC96663B-F29E-4A56-9623-DFE3C9145510}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="375" yWindow="3045" windowWidth="17280" windowHeight="11820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>Run Scenarios</t>
   </si>
@@ -103,6 +103,9 @@
   </si>
   <si>
     <t>Run optimal scenarios</t>
+  </si>
+  <si>
+    <t>Figure out why CO2 taxes not applied in 2025</t>
   </si>
 </sst>
 </file>
@@ -458,10 +461,12 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1"/>
+      <c r="B2" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
     </row>
@@ -474,7 +479,7 @@
       <c r="D3" s="1"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="1"/>

</xml_diff>

<commit_message>
add specific C tax in 2025-30.
</commit_message>
<xml_diff>
--- a/tasks.xlsx
+++ b/tasks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\GCAM-CDR-policy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC96663B-F29E-4A56-9623-DFE3C9145510}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6284267F-0E25-43E5-930C-FC522BF54423}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="375" yWindow="3045" windowWidth="17280" windowHeight="11820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7980" yWindow="5460" windowWidth="17280" windowHeight="11820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>Run Scenarios</t>
   </si>
@@ -106,6 +106,9 @@
   </si>
   <si>
     <t>Figure out why CO2 taxes not applied in 2025</t>
+  </si>
+  <si>
+    <t>but…... No C tax in 25/30…. Probably need to find data for and implement a flat tax….</t>
   </si>
 </sst>
 </file>
@@ -136,7 +139,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
+        <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -482,7 +485,9 @@
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="1"/>
+      <c r="B4" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
     </row>

</xml_diff>

<commit_message>
recreate output data for 3 no cost decrease baselines
</commit_message>
<xml_diff>
--- a/tasks.xlsx
+++ b/tasks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\GCAM-CDR-policy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57E3F617-F9A0-41BA-A31B-135ACCDD3194}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA36488D-20AB-4704-A9F9-FF4D7A019DA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7980" yWindow="5460" windowWidth="17280" windowHeight="11820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -112,7 +112,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -131,6 +131,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -144,10 +150,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -446,25 +453,25 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="1"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="1"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="1"/>
@@ -476,12 +483,12 @@
       <c r="B6" s="1"/>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="A8" s="3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -491,7 +498,7 @@
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="A13" s="3" t="s">
         <v>19</v>
       </c>
     </row>
@@ -501,7 +508,7 @@
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="A16" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -511,7 +518,7 @@
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+      <c r="A18" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
3/8 subsidy no CR
</commit_message>
<xml_diff>
--- a/tasks.xlsx
+++ b/tasks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\GCAM-CDR-policy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{236C0A1D-C75C-42ED-9BB2-31BF00A41B4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BB4DFB8-35C1-4066-AD5E-62F7783BB1A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="60" yWindow="1635" windowWidth="28740" windowHeight="13845" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -210,7 +210,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -229,6 +229,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -242,10 +248,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -670,12 +677,12 @@
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+      <c r="A28" s="2" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+      <c r="A29" s="2" t="s">
         <v>33</v>
       </c>
     </row>
@@ -695,7 +702,7 @@
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34" s="1" t="s">
+      <c r="A34" s="3" t="s">
         <v>52</v>
       </c>
     </row>

</xml_diff>